<commit_message>
update tests after supplier commented in init data file
</commit_message>
<xml_diff>
--- a/fmt/tests/condominium_import.xlsx
+++ b/fmt/tests/condominium_import.xlsx
@@ -562,76 +562,80 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -950,128 +954,128 @@
   <dimension ref="A1:R2"/>
   <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.59"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="14.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="17.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="9.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="9.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="21.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="18.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="17.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="17.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="14.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="21.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="14.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="17.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="9.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="21.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="18.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="17.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="17.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="14.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="21.88"/>
   </cols>
   <sheetData>
-    <row r="1" s="4" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" s="5" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="R1" s="4" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="0" t="n">
+      <c r="E2" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="0" t="n">
+      <c r="H2" s="1" t="n">
         <v>1083</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="L2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="M2" s="0" t="n">
+      <c r="L2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="N2" s="7" t="n">
+      <c r="N2" s="8" t="n">
         <v>44743</v>
       </c>
-      <c r="O2" s="7" t="n">
+      <c r="O2" s="8" t="n">
         <v>45107</v>
       </c>
-      <c r="P2" s="6" t="s">
+      <c r="P2" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="Q2" s="6" t="s">
+      <c r="Q2" s="7" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1096,41 +1100,41 @@
   <dimension ref="A1:C23"/>
   <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="23.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.13"/>
   </cols>
   <sheetData>
-    <row r="1" s="10" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="10" t="s">
+    <row r="1" s="11" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="C2" s="0" t="n">
+      <c r="C2" s="1" t="n">
         <v>1000</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="0" t="s">
+      <c r="A3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="C3" s="0" t="n">
+      <c r="C3" s="1" t="n">
         <v>1000</v>
       </c>
     </row>
@@ -1157,217 +1161,217 @@
   <dimension ref="A1:C19"/>
   <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.15"/>
   </cols>
   <sheetData>
-    <row r="1" s="8" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="8" t="s">
+    <row r="1" s="9" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="9" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="B2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" s="0" t="n">
+      <c r="B2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="n">
         <v>163</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="0" t="n">
+      <c r="C3" s="1" t="n">
         <v>163</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C4" s="0" t="n">
+      <c r="C4" s="1" t="n">
         <v>124</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C5" s="0" t="n">
+      <c r="C5" s="1" t="n">
         <v>124</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C6" s="0" t="n">
+      <c r="C6" s="1" t="n">
         <v>263</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C7" s="0" t="n">
+      <c r="C7" s="1" t="n">
         <v>64</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="B8" s="0" t="n">
+      <c r="B8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C8" s="0" t="n">
+      <c r="C8" s="1" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="B9" s="0" t="n">
+      <c r="B9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C9" s="0" t="n">
+      <c r="C9" s="1" t="n">
         <v>19</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="B10" s="0" t="n">
+      <c r="B10" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="C10" s="0" t="n">
+      <c r="C10" s="1" t="n">
         <v>64</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="B11" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" s="0" t="n">
+      <c r="A11" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="1" t="n">
         <v>163</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="B12" s="0" t="n">
+      <c r="A12" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="0" t="n">
+      <c r="C12" s="1" t="n">
         <v>163</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="B13" s="0" t="n">
+      <c r="A13" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="0" t="n">
+      <c r="C13" s="1" t="n">
         <v>124</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="B14" s="0" t="n">
+      <c r="A14" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C14" s="0" t="n">
+      <c r="C14" s="1" t="n">
         <v>124</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="B15" s="0" t="n">
+      <c r="A15" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C15" s="0" t="n">
+      <c r="C15" s="1" t="n">
         <v>263</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="B16" s="0" t="n">
+      <c r="A16" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B16" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C16" s="0" t="n">
+      <c r="C16" s="1" t="n">
         <v>64</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="B17" s="0" t="n">
+      <c r="A17" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B17" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C17" s="0" t="n">
+      <c r="C17" s="1" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="B18" s="0" t="n">
+      <c r="A18" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B18" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C18" s="0" t="n">
+      <c r="C18" s="1" t="n">
         <v>19</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="B19" s="0" t="n">
+      <c r="A19" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="C19" s="0" t="n">
+      <c r="C19" s="1" t="n">
         <v>64</v>
       </c>
     </row>
@@ -1390,104 +1394,82 @@
   <dimension ref="A1:A26"/>
   <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.26"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="2" s="17" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="n">
+    <row r="2" s="18" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="18" t="n">
         <v>1003</v>
       </c>
     </row>
-    <row r="3" s="17" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="17" t="n">
-        <v>1012</v>
-      </c>
-    </row>
-    <row r="4" s="17" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17" t="n">
-        <v>1020</v>
-      </c>
-    </row>
-    <row r="5" s="17" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17" t="n">
-        <v>1049</v>
-      </c>
-    </row>
-    <row r="6" s="17" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17" t="n">
-        <v>1090</v>
-      </c>
-    </row>
+    <row r="3" s="18" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" s="18" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" s="18" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" s="18" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17" t="n">
-        <v>1097</v>
-      </c>
+      <c r="A7" s="18"/>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="n">
-        <v>1129</v>
-      </c>
+      <c r="A8" s="18"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17" t="n">
-        <v>1131</v>
-      </c>
+      <c r="A9" s="18"/>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17"/>
+      <c r="A10" s="18"/>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17"/>
+      <c r="A11" s="18"/>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17"/>
+      <c r="A12" s="18"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="17"/>
+      <c r="A13" s="18"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17"/>
+      <c r="A14" s="18"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17"/>
+      <c r="A15" s="18"/>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17"/>
+      <c r="A16" s="18"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17"/>
+      <c r="A17" s="18"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17"/>
+      <c r="A18" s="18"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17"/>
+      <c r="A19" s="18"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17"/>
+      <c r="A20" s="18"/>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17"/>
+      <c r="A21" s="18"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="17"/>
+      <c r="A22" s="18"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17"/>
+      <c r="A23" s="18"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="17"/>
+      <c r="A24" s="18"/>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="17"/>
+      <c r="A25" s="18"/>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="17"/>
+      <c r="A26" s="18"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:A26">
@@ -1511,51 +1493,51 @@
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="23.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="23.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="23.4"/>
   </cols>
   <sheetData>
-    <row r="1" s="4" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" s="5" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="1" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1581,73 +1563,73 @@
   <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="I1" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="J1" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="K1" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="L1" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="M1" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="N1" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="O1" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="P1" s="9" t="s">
+      <c r="P1" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="Q1" s="9" t="s">
+      <c r="Q1" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="R1" s="9" t="s">
+      <c r="R1" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="S1" s="10" t="s">
+      <c r="S1" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="T1" s="10" t="s">
+      <c r="T1" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="U1" s="10" t="s">
+      <c r="U1" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="V1" s="10" t="s">
+      <c r="V1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="W1" s="10" t="s">
+      <c r="W1" s="11" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1670,290 +1652,290 @@
   <dimension ref="A1:W6"/>
   <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="25.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="22.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="16.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="16.59"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="27.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="18.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="17" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="15.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="22.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="21.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="17.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="23.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="25.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="22.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="16.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="1" width="16.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="27.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="18.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="17" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="15.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="22.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="21.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="17.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="23.4"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="J1" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="K1" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="L1" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="M1" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="N1" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="O1" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="P1" s="9" t="s">
+      <c r="P1" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="Q1" s="9" t="s">
+      <c r="Q1" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="R1" s="9" t="s">
+      <c r="R1" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="S1" s="10" t="s">
+      <c r="S1" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="T1" s="10" t="s">
+      <c r="T1" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="U1" s="10" t="s">
+      <c r="U1" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="V1" s="10" t="s">
+      <c r="V1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="W1" s="10" t="s">
+      <c r="W1" s="11" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="0" t="s">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="G2" s="0" t="n">
+      <c r="G2" s="1" t="n">
         <v>1083</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="H2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="I2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J2" s="0" t="s">
+      <c r="J2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="M2" s="6" t="s">
+      <c r="M2" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="O2" s="6" t="s">
+      <c r="O2" s="7" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G3" s="0" t="n">
+      <c r="G3" s="1" t="n">
         <v>9880</v>
       </c>
-      <c r="H3" s="0" t="s">
+      <c r="H3" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="I3" s="0" t="s">
+      <c r="I3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J3" s="0" t="s">
+      <c r="J3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="M3" s="6" t="s">
+      <c r="M3" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="O3" s="6" t="s">
+      <c r="O3" s="7" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="G4" s="0" t="n">
+      <c r="G4" s="1" t="n">
         <v>1083</v>
       </c>
-      <c r="H4" s="0" t="s">
+      <c r="H4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I4" s="0" t="s">
+      <c r="I4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="0" t="s">
+      <c r="J4" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="M4" s="6" t="s">
+      <c r="M4" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="O4" s="6" t="s">
+      <c r="O4" s="7" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="G5" s="0" t="n">
+      <c r="G5" s="1" t="n">
         <v>1083</v>
       </c>
-      <c r="H5" s="0" t="s">
+      <c r="H5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="0" t="s">
+      <c r="I5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J5" s="0" t="s">
+      <c r="J5" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="K5" s="6" t="s">
+      <c r="K5" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="M5" s="12" t="s">
+      <c r="M5" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="O5" s="6" t="s">
+      <c r="O5" s="7" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="F6" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="G6" s="0" t="n">
+      <c r="G6" s="1" t="n">
         <v>1083</v>
       </c>
-      <c r="H6" s="0" t="s">
+      <c r="H6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I6" s="0" t="s">
+      <c r="I6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J6" s="0" t="s">
+      <c r="J6" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="K6" s="6" t="s">
+      <c r="K6" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="M6" s="12" t="s">
+      <c r="M6" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="O6" s="12" t="s">
+      <c r="O6" s="13" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1982,108 +1964,108 @@
   <dimension ref="A1:H6"/>
   <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="23.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="23.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="31.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="23.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="23.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="31.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="23"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="F1" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="G1" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="11" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="0" t="n">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" s="0" t="n">
+      <c r="C3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C4" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" s="0" t="n">
+      <c r="C4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="1" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C5" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" s="0" t="n">
+      <c r="C5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="1" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C6" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" s="0" t="n">
+      <c r="C6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="1" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2108,151 +2090,151 @@
   <dimension ref="A1:G6"/>
   <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="23.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="27.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="21.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="48.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="27.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="21.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="48.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16.26"/>
   </cols>
   <sheetData>
-    <row r="1" s="10" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="10" t="s">
+    <row r="1" s="11" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="11" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="0" t="s">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="1" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="G3" s="1" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="G4" s="1" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="G5" s="1" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="F6" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="G6" s="0" t="s">
+      <c r="G6" s="1" t="s">
         <v>101</v>
       </c>
     </row>
@@ -2277,51 +2259,51 @@
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12.73"/>
   </cols>
   <sheetData>
-    <row r="1" s="10" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="10" t="s">
+    <row r="1" s="11" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="10" t="s">
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="11" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="0" t="s">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="1" t="n">
         <v>1083</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="1" t="s">
         <v>23</v>
       </c>
     </row>
@@ -2344,252 +2326,252 @@
   <dimension ref="A1:J15"/>
   <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="0" width="17.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="23.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="1" width="17.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="20.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="23.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="14" t="s">
         <v>102</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="14" t="s">
         <v>103</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="I1" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="J1" s="14" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="0" t="s">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D7" s="0" t="n">
+      <c r="D7" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
+      <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D8" s="0" t="n">
+      <c r="D8" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+      <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="D9" s="0" t="n">
+      <c r="D9" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="n">
+      <c r="A10" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="D10" s="0" t="n">
+      <c r="D10" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="n">
+      <c r="A11" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D11" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" s="0" t="n">
+      <c r="D11" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="n">
+      <c r="A12" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D12" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="I12" s="0" t="n">
+      <c r="D12" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="n">
+      <c r="A13" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D13" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" s="0" t="n">
+      <c r="D13" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="1" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="n">
+      <c r="A14" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D14" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="I14" s="0" t="n">
+      <c r="D14" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="1" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="n">
+      <c r="A15" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D15" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="I15" s="0" t="n">
+      <c r="D15" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="1" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2614,181 +2596,181 @@
   <dimension ref="A1:D15"/>
   <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.4"/>
   </cols>
   <sheetData>
-    <row r="1" s="10" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="10" t="s">
+    <row r="1" s="11" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="0" t="n">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C2" s="15" t="n">
+      <c r="C2" s="16" t="n">
         <v>44743</v>
       </c>
-      <c r="D2" s="15"/>
+      <c r="D2" s="16"/>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C3" s="15" t="n">
+      <c r="C3" s="16" t="n">
         <v>44743</v>
       </c>
-      <c r="D3" s="15"/>
+      <c r="D3" s="16"/>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C4" s="15" t="n">
+      <c r="C4" s="16" t="n">
         <v>44743</v>
       </c>
-      <c r="D4" s="15"/>
+      <c r="D4" s="16"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C5" s="15" t="n">
+      <c r="C5" s="16" t="n">
         <v>44743</v>
       </c>
-      <c r="D5" s="15"/>
+      <c r="D5" s="16"/>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="16" t="n">
         <v>44743</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="C7" s="16" t="n">
         <v>44743</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
+      <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="0" t="n">
+      <c r="B8" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="15" t="n">
+      <c r="C8" s="16" t="n">
         <v>44743</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+      <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="0" t="n">
+      <c r="B9" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="16" t="n">
         <v>44743</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="n">
+      <c r="A10" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="0" t="n">
+      <c r="B10" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="16" t="n">
         <v>44743</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="n">
+      <c r="A11" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="0" t="n">
+      <c r="B11" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C11" s="15" t="n">
+      <c r="C11" s="16" t="n">
         <v>44743</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="n">
+      <c r="A12" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="0" t="n">
+      <c r="B12" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="15" t="n">
+      <c r="C12" s="16" t="n">
         <v>44743</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="n">
+      <c r="A13" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="0" t="n">
+      <c r="B13" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C13" s="15" t="n">
+      <c r="C13" s="16" t="n">
         <v>44743</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="n">
+      <c r="A14" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="0" t="n">
+      <c r="B14" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C14" s="15" t="n">
+      <c r="C14" s="16" t="n">
         <v>44743</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="n">
+      <c r="A15" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="0" t="n">
+      <c r="B15" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C15" s="15" t="n">
+      <c r="C15" s="16" t="n">
         <v>44743</v>
       </c>
     </row>

</xml_diff>